<commit_message>
added stream test scene
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Relics.xlsx
+++ b/Assets/StreamingAssets/Configurations/Relics.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E5A6B2-A815-4D9F-A547-72FAC12E4D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480" activeTab="2"/>
+    <workbookView xWindow="11985" yWindow="5430" windowWidth="25575" windowHeight="13665" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingRelicConditions" sheetId="1" r:id="rId1"/>
@@ -626,361 +632,25 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -997,315 +667,28 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1563,22 +946,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.18333333333333" customWidth="1"/>
-    <col min="2" max="2" width="11.725" customWidth="1"/>
-    <col min="3" max="3" width="15.45" customWidth="1"/>
-    <col min="4" max="4" width="28.725" customWidth="1"/>
-    <col min="5" max="5" width="14.725" customWidth="1"/>
-    <col min="6" max="6" width="13.45" customWidth="1"/>
-    <col min="7" max="7" width="10.45" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1764,7 +1147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="1" spans="1:7">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1784,7 +1167,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" customFormat="1" spans="1:7">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1804,7 +1187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="1" spans="1:7">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1824,7 +1207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="1" spans="1:7">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1886,36 +1269,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.41666666666667" customWidth="1"/>
-    <col min="2" max="2" width="13.5416666666667" customWidth="1"/>
-    <col min="3" max="3" width="25.45" customWidth="1"/>
-    <col min="4" max="4" width="12.1833333333333" customWidth="1"/>
-    <col min="5" max="5" width="5.45" customWidth="1"/>
-    <col min="6" max="6" width="20.1833333333333" customWidth="1"/>
-    <col min="7" max="7" width="3.81666666666667" customWidth="1"/>
-    <col min="8" max="8" width="7.45" customWidth="1"/>
-    <col min="9" max="9" width="10.2666666666667" customWidth="1"/>
-    <col min="10" max="10" width="13.1833333333333" customWidth="1"/>
-    <col min="11" max="11" width="17.1833333333333" customWidth="1"/>
-    <col min="12" max="12" width="14.1833333333333" customWidth="1"/>
-    <col min="13" max="13" width="12.45" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.42578125" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="3.85546875" customWidth="1"/>
+    <col min="8" max="8" width="7.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" customWidth="1"/>
+    <col min="11" max="11" width="17.140625" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.42578125" customWidth="1"/>
     <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="11.8166666666667" customWidth="1"/>
-    <col min="16" max="16" width="11.5416666666667" customWidth="1"/>
-    <col min="17" max="17" width="17.1833333333333" customWidth="1"/>
+    <col min="15" max="15" width="11.85546875" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" spans="1:18">
+    <row r="1" spans="1:18" ht="30">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1971,7 +1352,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:18">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2003,7 +1384,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:18">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2035,7 +1416,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:18">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2067,7 +1448,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:18">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2099,7 +1480,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:18">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2131,7 +1512,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:18">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2163,7 +1544,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:18">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2195,7 +1576,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:18">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2227,7 +1608,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:18">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2259,7 +1640,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:18">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2291,7 +1672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:18">
       <c r="A12">
         <v>10</v>
       </c>
@@ -2320,7 +1701,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:18">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2349,7 +1730,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:18">
       <c r="A14">
         <v>12</v>
       </c>
@@ -2374,8 +1755,11 @@
       <c r="J14">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="K14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18">
       <c r="A15">
         <v>13</v>
       </c>
@@ -2400,8 +1784,11 @@
       <c r="J15">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:10">
+      <c r="K15">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18">
       <c r="A16">
         <v>14</v>
       </c>
@@ -2426,8 +1813,11 @@
       <c r="J16">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:10">
+      <c r="K16">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17">
         <v>15</v>
       </c>
@@ -2452,8 +1842,11 @@
       <c r="J17">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:10">
+      <c r="K17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18">
         <v>16</v>
       </c>
@@ -2478,8 +1871,11 @@
       <c r="J18">
         <v>4</v>
       </c>
-    </row>
-    <row r="19" spans="1:10">
+      <c r="K18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19">
         <v>17</v>
       </c>
@@ -2504,8 +1900,11 @@
       <c r="J19">
         <v>4</v>
       </c>
-    </row>
-    <row r="20" spans="1:10">
+      <c r="K19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20">
         <v>18</v>
       </c>
@@ -2530,8 +1929,11 @@
       <c r="J20">
         <v>4</v>
       </c>
-    </row>
-    <row r="21" spans="1:10">
+      <c r="K20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21">
         <v>19</v>
       </c>
@@ -2556,8 +1958,11 @@
       <c r="J21">
         <v>4</v>
       </c>
-    </row>
-    <row r="22" spans="1:10">
+      <c r="K21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22">
         <v>20</v>
       </c>
@@ -2582,8 +1987,11 @@
       <c r="J22">
         <v>4</v>
       </c>
-    </row>
-    <row r="23" spans="1:10">
+      <c r="K22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23">
         <v>21</v>
       </c>
@@ -2608,8 +2016,11 @@
       <c r="J23">
         <v>25</v>
       </c>
-    </row>
-    <row r="24" spans="1:10">
+      <c r="K23">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24">
         <v>22</v>
       </c>
@@ -2637,8 +2048,11 @@
       <c r="J24">
         <v>2</v>
       </c>
-    </row>
-    <row r="25" spans="1:10">
+      <c r="K24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
       <c r="A25">
         <v>23</v>
       </c>
@@ -2666,8 +2080,11 @@
       <c r="J25">
         <v>4</v>
       </c>
-    </row>
-    <row r="26" spans="1:10">
+      <c r="K25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26">
         <v>24</v>
       </c>
@@ -2695,8 +2112,11 @@
       <c r="J26">
         <v>3</v>
       </c>
-    </row>
-    <row r="27" spans="1:10">
+      <c r="K26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
       <c r="A27">
         <v>25</v>
       </c>
@@ -2724,8 +2144,11 @@
       <c r="J27">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="1:10">
+      <c r="K27">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28">
         <v>26</v>
       </c>
@@ -2753,8 +2176,11 @@
       <c r="J28">
         <v>5</v>
       </c>
-    </row>
-    <row r="29" spans="1:10">
+      <c r="K28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
       <c r="A29">
         <v>27</v>
       </c>
@@ -2782,8 +2208,11 @@
       <c r="J29">
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="1:10">
+      <c r="K29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="A30">
         <v>28</v>
       </c>
@@ -2811,8 +2240,11 @@
       <c r="J30">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="1:10">
+      <c r="K30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31">
         <v>29</v>
       </c>
@@ -2840,8 +2272,11 @@
       <c r="J31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:10">
+      <c r="K31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
       <c r="A32">
         <v>30</v>
       </c>
@@ -2869,8 +2304,11 @@
       <c r="J32">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="33" spans="1:10">
+      <c r="K32">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
       <c r="A33">
         <v>31</v>
       </c>
@@ -2898,8 +2336,11 @@
       <c r="J33">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="34" spans="1:10">
+      <c r="K33">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
       <c r="A34">
         <v>32</v>
       </c>
@@ -2927,8 +2368,11 @@
       <c r="J34">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="35" spans="1:10">
+      <c r="K34">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
       <c r="A35">
         <v>33</v>
       </c>
@@ -2953,8 +2397,11 @@
       <c r="J35">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="36" spans="1:10">
+      <c r="K35">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36">
         <v>34</v>
       </c>
@@ -2979,8 +2426,11 @@
       <c r="J36">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:10">
+      <c r="K36">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
       <c r="A37">
         <v>35</v>
       </c>
@@ -3005,8 +2455,11 @@
       <c r="J37">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="38" spans="1:10">
+      <c r="K37">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
       <c r="A38">
         <v>36</v>
       </c>
@@ -3031,8 +2484,11 @@
       <c r="J38">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="39" spans="1:10">
+      <c r="K38">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
       <c r="A39">
         <v>37</v>
       </c>
@@ -3057,8 +2513,11 @@
       <c r="J39">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="40" spans="1:10">
+      <c r="K39">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40">
         <v>38</v>
       </c>
@@ -3083,8 +2542,11 @@
       <c r="J40">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="41" spans="1:10">
+      <c r="K40">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
       <c r="A41">
         <v>39</v>
       </c>
@@ -3112,8 +2574,11 @@
       <c r="J41">
         <v>5</v>
       </c>
-    </row>
-    <row r="42" spans="1:10">
+      <c r="K41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
       <c r="A42">
         <v>40</v>
       </c>
@@ -3141,8 +2606,11 @@
       <c r="J42">
         <v>5</v>
       </c>
-    </row>
-    <row r="43" spans="1:10">
+      <c r="K42">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
       <c r="A43">
         <v>41</v>
       </c>
@@ -3170,8 +2638,11 @@
       <c r="J43">
         <v>5</v>
       </c>
-    </row>
-    <row r="44" spans="1:10">
+      <c r="K43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
       <c r="A44">
         <v>42</v>
       </c>
@@ -3196,8 +2667,11 @@
       <c r="J44">
         <v>5</v>
       </c>
-    </row>
-    <row r="45" spans="1:10">
+      <c r="K44">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
       <c r="A45">
         <v>43</v>
       </c>
@@ -3222,8 +2696,11 @@
       <c r="J45">
         <v>5</v>
       </c>
-    </row>
-    <row r="46" spans="1:10">
+      <c r="K45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
       <c r="A46">
         <v>44</v>
       </c>
@@ -3248,6 +2725,9 @@
       <c r="J46">
         <v>5</v>
       </c>
+      <c r="K46">
+        <v>5</v>
+      </c>
     </row>
     <row r="47" spans="1:14">
       <c r="A47">
@@ -3274,6 +2754,9 @@
       <c r="J47">
         <v>500</v>
       </c>
+      <c r="K47">
+        <v>500</v>
+      </c>
       <c r="L47">
         <v>16</v>
       </c>
@@ -3286,24 +2769,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M14"/>
-  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="23.5416666666667" customWidth="1"/>
-    <col min="4" max="7" width="18.1833333333333" customWidth="1"/>
-    <col min="8" max="8" width="10.5416666666667" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" customWidth="1"/>
+    <col min="4" max="7" width="18.140625" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="12.8166666666667" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" customWidth="1"/>
     <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="11.2666666666667" customWidth="1"/>
-    <col min="13" max="13" width="10.725" customWidth="1"/>
+    <col min="12" max="12" width="11.28515625" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -3347,7 +2828,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:13">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3376,7 +2857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:13">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3405,7 +2886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:13">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3434,7 +2915,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:13">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3463,7 +2944,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:13">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3492,7 +2973,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" ht="42" spans="1:13">
+    <row r="7" spans="1:13" ht="60">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3533,7 +3014,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="28" spans="1:11">
+    <row r="8" spans="1:13" ht="30">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3565,7 +3046,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="42" spans="1:11">
+    <row r="9" spans="1:13" ht="45">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3600,7 +3081,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:13">
       <c r="A10">
         <v>8</v>
       </c>
@@ -3632,7 +3113,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:13">
       <c r="A11">
         <v>9</v>
       </c>
@@ -3667,7 +3148,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:13">
       <c r="A12">
         <v>10</v>
       </c>
@@ -3696,7 +3177,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:13">
       <c r="A13">
         <v>11</v>
       </c>
@@ -3725,12 +3206,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="6:7">
+    <row r="14" spans="1:13">
       <c r="F14" s="1"/>
-      <c r="G14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>